<commit_message>
feat: add animated hero box, marketplace sample files, and reconcile tests
</commit_message>
<xml_diff>
--- a/sample-data/meesho-settlement-sample.xlsx
+++ b/sample-data/meesho-settlement-sample.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M38"/>
+  <dimension ref="A1:M24"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -442,37 +442,37 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2345891101</v>
+        <v>MH1001</v>
       </c>
       <c r="B2" t="str">
-        <v>TXN891101JUL26</v>
+        <v>TXNH1001JUL26</v>
       </c>
       <c r="C2" t="str">
         <v>03/07/2026</v>
       </c>
       <c r="D2" t="str">
-        <v>WMN-KRT-YLW-XL</v>
+        <v>SAR-BNJ-RED</v>
       </c>
       <c r="E2" t="str">
-        <v>Womens Rayon Kurti - Yellow XL</v>
+        <v>Banarasi Silk Saree - Red</v>
       </c>
       <c r="F2">
-        <v>549</v>
+        <v>1199</v>
       </c>
       <c r="G2">
-        <v>45.04</v>
+        <v>85.34</v>
       </c>
       <c r="H2">
-        <v>48.8</v>
+        <v>41.17</v>
       </c>
       <c r="I2">
         <v>0</v>
       </c>
       <c r="J2">
-        <v>0.55</v>
+        <v>1.2</v>
       </c>
       <c r="K2">
-        <v>454.61</v>
+        <v>1071.29</v>
       </c>
       <c r="L2" t="str">
         <v>Delivered</v>
@@ -483,37 +483,37 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2345891102</v>
+        <v>MH1002</v>
       </c>
       <c r="B3" t="str">
-        <v>TXN891102JUL26</v>
+        <v>TXNH1002JUL26</v>
       </c>
       <c r="C3" t="str">
         <v>05/07/2026</v>
       </c>
       <c r="D3" t="str">
-        <v>FTW-SLPR-BLU-9</v>
+        <v>KDS-GRL-FRK-5Y</v>
       </c>
       <c r="E3" t="str">
-        <v>Mens Casual Slippers Blue Size 9</v>
+        <v>Kids Girls Party Frock, Age 5Y</v>
       </c>
       <c r="F3">
-        <v>349</v>
+        <v>429</v>
       </c>
       <c r="G3">
-        <v>32.64</v>
+        <v>37.6</v>
       </c>
       <c r="H3">
-        <v>51.48</v>
+        <v>49.1</v>
       </c>
       <c r="I3">
         <v>0</v>
       </c>
       <c r="J3">
-        <v>0.35</v>
+        <v>0.43</v>
       </c>
       <c r="K3">
-        <v>264.53</v>
+        <v>341.87</v>
       </c>
       <c r="L3" t="str">
         <v>Delivered</v>
@@ -524,40 +524,40 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2345891103</v>
+        <v>MH1003</v>
       </c>
       <c r="B4" t="str">
-        <v>TXN891103JUL26</v>
+        <v>TXNH1003JUL26</v>
       </c>
       <c r="C4" t="str">
         <v>07/07/2026</v>
       </c>
       <c r="D4" t="str">
-        <v>ACC-WTCH-BLK</v>
+        <v>KDS-GRL-FRK-5Y</v>
       </c>
       <c r="E4" t="str">
-        <v>Analog Wrist Watch - Black Dial</v>
+        <v>Kids Girls Party Frock, Age 5Y</v>
       </c>
       <c r="F4">
-        <v>399</v>
+        <v>429</v>
       </c>
       <c r="G4">
-        <v>35.74</v>
+        <v>37.6</v>
       </c>
       <c r="H4">
-        <v>51.34</v>
+        <v>0</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="J4">
-        <v>0.4</v>
+        <v>0.43</v>
       </c>
       <c r="K4">
-        <v>292.52</v>
+        <v>322.97</v>
       </c>
       <c r="L4" t="str">
-        <v>Delivered</v>
+        <v>RTO</v>
       </c>
       <c r="M4" t="str">
         <v>Done</v>
@@ -565,37 +565,37 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2345891104</v>
+        <v>MH1004</v>
       </c>
       <c r="B5" t="str">
-        <v>TXN891104JUL26</v>
+        <v>TXNH1004JUL26</v>
       </c>
       <c r="C5" t="str">
         <v>09/07/2026</v>
       </c>
       <c r="D5" t="str">
-        <v>WMN-KRT-YLW-XL</v>
+        <v>FTW-SLPR-BLU-9</v>
       </c>
       <c r="E5" t="str">
-        <v>Womens Rayon Kurti - Yellow XL</v>
+        <v>Mens Casual Slippers Blue Size 9</v>
       </c>
       <c r="F5">
-        <v>549</v>
+        <v>349</v>
       </c>
       <c r="G5">
-        <v>45.04</v>
+        <v>32.64</v>
       </c>
       <c r="H5">
-        <v>43.28</v>
+        <v>53.36</v>
       </c>
       <c r="I5">
         <v>0</v>
       </c>
       <c r="J5">
-        <v>0.55</v>
+        <v>0.35</v>
       </c>
       <c r="K5">
-        <v>460.13</v>
+        <v>262.65</v>
       </c>
       <c r="L5" t="str">
         <v>Delivered</v>
@@ -606,37 +606,37 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2345891105</v>
+        <v>MH1005</v>
       </c>
       <c r="B6" t="str">
-        <v>TXN891105JUL26</v>
+        <v>TXNH1005JUL26</v>
       </c>
       <c r="C6" t="str">
         <v>11/07/2026</v>
       </c>
       <c r="D6" t="str">
-        <v>KRT-WT-MENS-L</v>
+        <v>WMN-KRT-YLW-XL</v>
       </c>
       <c r="E6" t="str">
-        <v>Cotton Kurta Set - White, Men L</v>
+        <v>Womens Rayon Kurti - Yellow XL</v>
       </c>
       <c r="F6">
-        <v>749</v>
+        <v>549</v>
       </c>
       <c r="G6">
-        <v>57.44</v>
+        <v>45.04</v>
       </c>
       <c r="H6">
-        <v>44.39</v>
+        <v>42.48</v>
       </c>
       <c r="I6">
         <v>0</v>
       </c>
       <c r="J6">
-        <v>0.75</v>
+        <v>0.55</v>
       </c>
       <c r="K6">
-        <v>646.42</v>
+        <v>427.93</v>
       </c>
       <c r="L6" t="str">
         <v>Delivered</v>
@@ -647,40 +647,40 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2345891107</v>
+        <v>MH1006</v>
       </c>
       <c r="B7" t="str">
-        <v>TXN891107JUL26</v>
+        <v>TXNH1006JUL26</v>
       </c>
       <c r="C7" t="str">
-        <v>15/07/2026</v>
+        <v>13/07/2026</v>
       </c>
       <c r="D7" t="str">
-        <v>HOM-BDSHT-DBL</v>
+        <v>FTW-SLPR-BLU-9</v>
       </c>
       <c r="E7" t="str">
-        <v>Double Bedsheet with 2 Pillow Covers</v>
+        <v>Mens Casual Slippers Blue Size 9</v>
       </c>
       <c r="F7">
-        <v>649</v>
+        <v>349</v>
       </c>
       <c r="G7">
-        <v>51.24</v>
+        <v>32.64</v>
       </c>
       <c r="H7">
-        <v>51.07</v>
+        <v>49.77</v>
       </c>
       <c r="I7">
         <v>0</v>
       </c>
       <c r="J7">
-        <v>0.65</v>
+        <v>0.35</v>
       </c>
       <c r="K7">
-        <v>546.04</v>
+        <v>266.24</v>
       </c>
       <c r="L7" t="str">
-        <v>Return</v>
+        <v>Delivered</v>
       </c>
       <c r="M7" t="str">
         <v>Done</v>
@@ -688,37 +688,37 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2345891108</v>
+        <v>MH1008</v>
       </c>
       <c r="B8" t="str">
-        <v>TXN891108JUL26</v>
+        <v>TXNH1008JUL26</v>
       </c>
       <c r="C8" t="str">
         <v>17/07/2026</v>
       </c>
       <c r="D8" t="str">
-        <v>KDS-GRL-FRK-5Y</v>
+        <v>KRT-WT-MENS-L</v>
       </c>
       <c r="E8" t="str">
-        <v>Kids Girls Party Frock, Age 5Y</v>
+        <v>Cotton Kurta Set - White, Men L</v>
       </c>
       <c r="F8">
-        <v>429</v>
+        <v>749</v>
       </c>
       <c r="G8">
-        <v>37.6</v>
+        <v>57.44</v>
       </c>
       <c r="H8">
-        <v>44.84</v>
+        <v>53.47</v>
       </c>
       <c r="I8">
         <v>0</v>
       </c>
       <c r="J8">
-        <v>0.43</v>
+        <v>0.75</v>
       </c>
       <c r="K8">
-        <v>346.13</v>
+        <v>637.34</v>
       </c>
       <c r="L8" t="str">
         <v>Delivered</v>
@@ -729,37 +729,37 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2345891109</v>
+        <v>MH1009</v>
       </c>
       <c r="B9" t="str">
-        <v>TXN891109JUL26</v>
+        <v>TXNH1009JUL26</v>
       </c>
       <c r="C9" t="str">
         <v>19/07/2026</v>
       </c>
       <c r="D9" t="str">
-        <v>KRT-WT-MENS-L</v>
+        <v>HOM-BDSHT-DBL</v>
       </c>
       <c r="E9" t="str">
-        <v>Cotton Kurta Set - White, Men L</v>
+        <v>Double Bedsheet with 2 Pillow Covers</v>
       </c>
       <c r="F9">
-        <v>749</v>
+        <v>649</v>
       </c>
       <c r="G9">
-        <v>57.44</v>
+        <v>51.24</v>
       </c>
       <c r="H9">
-        <v>54.49</v>
+        <v>47.98</v>
       </c>
       <c r="I9">
         <v>0</v>
       </c>
       <c r="J9">
-        <v>0.75</v>
+        <v>0.65</v>
       </c>
       <c r="K9">
-        <v>636.32</v>
+        <v>549.13</v>
       </c>
       <c r="L9" t="str">
         <v>Delivered</v>
@@ -770,10 +770,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2345891110</v>
+        <v>MH1010</v>
       </c>
       <c r="B10" t="str">
-        <v>TXN891110JUL26</v>
+        <v>TXNH1010JUL26</v>
       </c>
       <c r="C10" t="str">
         <v>21/07/2026</v>
@@ -791,7 +791,7 @@
         <v>35.74</v>
       </c>
       <c r="H10">
-        <v>53.6</v>
+        <v>50.65</v>
       </c>
       <c r="I10">
         <v>0</v>
@@ -800,7 +800,7 @@
         <v>0.4</v>
       </c>
       <c r="K10">
-        <v>309.26</v>
+        <v>312.21</v>
       </c>
       <c r="L10" t="str">
         <v>Delivered</v>
@@ -811,37 +811,37 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2345891111</v>
+        <v>MH1011</v>
       </c>
       <c r="B11" t="str">
-        <v>TXN891111JUL26</v>
+        <v>TXNH1011JUL26</v>
       </c>
       <c r="C11" t="str">
         <v>23/07/2026</v>
       </c>
       <c r="D11" t="str">
-        <v>MEN-TRS-DNM-32</v>
+        <v>ACC-WTCH-BLK</v>
       </c>
       <c r="E11" t="str">
-        <v>Mens Denim Jeans Slim Fit 32</v>
+        <v>Analog Wrist Watch - Black Dial</v>
       </c>
       <c r="F11">
-        <v>899</v>
+        <v>399</v>
       </c>
       <c r="G11">
-        <v>66.74</v>
+        <v>35.74</v>
       </c>
       <c r="H11">
-        <v>45.22</v>
+        <v>46.05</v>
       </c>
       <c r="I11">
         <v>0</v>
       </c>
       <c r="J11">
-        <v>0.9</v>
+        <v>0.4</v>
       </c>
       <c r="K11">
-        <v>770.14</v>
+        <v>316.81</v>
       </c>
       <c r="L11" t="str">
         <v>Delivered</v>
@@ -852,40 +852,40 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2345891112</v>
+        <v>MH1012</v>
       </c>
       <c r="B12" t="str">
-        <v>TXN891112JUL26</v>
+        <v>TXNH1012JUL26</v>
       </c>
       <c r="C12" t="str">
         <v>25/07/2026</v>
       </c>
       <c r="D12" t="str">
-        <v>ACC-WTCH-BLK</v>
+        <v>SAR-BNJ-RED</v>
       </c>
       <c r="E12" t="str">
-        <v>Analog Wrist Watch - Black Dial</v>
+        <v>Banarasi Silk Saree - Red</v>
       </c>
       <c r="F12">
-        <v>399</v>
+        <v>1199</v>
       </c>
       <c r="G12">
-        <v>35.74</v>
+        <v>85.34</v>
       </c>
       <c r="H12">
-        <v>0</v>
+        <v>47.86</v>
       </c>
       <c r="I12">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="J12">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="K12">
-        <v>226.86</v>
+        <v>1005.6</v>
       </c>
       <c r="L12" t="str">
-        <v>RTO</v>
+        <v>Delivered</v>
       </c>
       <c r="M12" t="str">
         <v>Done</v>
@@ -893,10 +893,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2345891113</v>
+        <v>MH1013</v>
       </c>
       <c r="B13" t="str">
-        <v>TXN891113JUL26</v>
+        <v>TXNH1013JUL26</v>
       </c>
       <c r="C13" t="str">
         <v>27/07/2026</v>
@@ -914,7 +914,7 @@
         <v>57.44</v>
       </c>
       <c r="H13">
-        <v>52.49</v>
+        <v>54.57</v>
       </c>
       <c r="I13">
         <v>0</v>
@@ -923,10 +923,10 @@
         <v>0.75</v>
       </c>
       <c r="K13">
-        <v>638.32</v>
+        <v>636.24</v>
       </c>
       <c r="L13" t="str">
-        <v>Delivered</v>
+        <v>Return</v>
       </c>
       <c r="M13" t="str">
         <v>Done</v>
@@ -934,40 +934,40 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2345891114</v>
+        <v>MH1014</v>
       </c>
       <c r="B14" t="str">
-        <v>TXN891114JUL26</v>
+        <v>TXNH1014JUL26</v>
       </c>
       <c r="C14" t="str">
         <v>29/07/2026</v>
       </c>
       <c r="D14" t="str">
-        <v>FTW-SLPR-BLU-9</v>
+        <v>KDS-GRL-FRK-5Y</v>
       </c>
       <c r="E14" t="str">
-        <v>Mens Casual Slippers Blue Size 9</v>
+        <v>Kids Girls Party Frock, Age 5Y</v>
       </c>
       <c r="F14">
-        <v>349</v>
+        <v>429</v>
       </c>
       <c r="G14">
-        <v>32.64</v>
+        <v>37.6</v>
       </c>
       <c r="H14">
-        <v>53.08</v>
+        <v>0</v>
       </c>
       <c r="I14">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="J14">
-        <v>0.35</v>
+        <v>0.43</v>
       </c>
       <c r="K14">
-        <v>262.93</v>
+        <v>322.97</v>
       </c>
       <c r="L14" t="str">
-        <v>Return</v>
+        <v>RTO</v>
       </c>
       <c r="M14" t="str">
         <v>Done</v>
@@ -975,37 +975,37 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2345891115</v>
+        <v>MH1015</v>
       </c>
       <c r="B15" t="str">
-        <v>TXN891115JUL26</v>
+        <v>TXNH1015JUL26</v>
       </c>
       <c r="C15" t="str">
         <v>02/07/2026</v>
       </c>
       <c r="D15" t="str">
-        <v>KRT-WT-MENS-L</v>
+        <v>HOM-BDSHT-DBL</v>
       </c>
       <c r="E15" t="str">
-        <v>Cotton Kurta Set - White, Men L</v>
+        <v>Double Bedsheet with 2 Pillow Covers</v>
       </c>
       <c r="F15">
-        <v>749</v>
+        <v>649</v>
       </c>
       <c r="G15">
-        <v>57.44</v>
+        <v>51.24</v>
       </c>
       <c r="H15">
-        <v>46.06</v>
+        <v>48.62</v>
       </c>
       <c r="I15">
         <v>0</v>
       </c>
       <c r="J15">
-        <v>0.75</v>
+        <v>0.65</v>
       </c>
       <c r="K15">
-        <v>644.75</v>
+        <v>548.49</v>
       </c>
       <c r="L15" t="str">
         <v>Delivered</v>
@@ -1016,37 +1016,37 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2345891116</v>
+        <v>MH1016</v>
       </c>
       <c r="B16" t="str">
-        <v>TXN891116JUL26</v>
+        <v>TXNH1016JUL26</v>
       </c>
       <c r="C16" t="str">
         <v>03/07/2026</v>
       </c>
       <c r="D16" t="str">
-        <v>HOM-BDSHT-DBL</v>
+        <v>KRT-WT-MENS-L</v>
       </c>
       <c r="E16" t="str">
-        <v>Double Bedsheet with 2 Pillow Covers</v>
+        <v>Cotton Kurta Set - White, Men L</v>
       </c>
       <c r="F16">
-        <v>649</v>
+        <v>749</v>
       </c>
       <c r="G16">
-        <v>51.24</v>
+        <v>57.44</v>
       </c>
       <c r="H16">
-        <v>41.84</v>
+        <v>42.36</v>
       </c>
       <c r="I16">
         <v>0</v>
       </c>
       <c r="J16">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="K16">
-        <v>555.27</v>
+        <v>648.45</v>
       </c>
       <c r="L16" t="str">
         <v>Delivered</v>
@@ -1057,37 +1057,37 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2345891117</v>
+        <v>MH1018</v>
       </c>
       <c r="B17" t="str">
-        <v>TXN891117JUL26</v>
+        <v>TXNH1018JUL26</v>
       </c>
       <c r="C17" t="str">
-        <v>05/07/2026</v>
+        <v>07/07/2026</v>
       </c>
       <c r="D17" t="str">
-        <v>KDS-GRL-FRK-5Y</v>
+        <v>FTW-SLPR-BLU-9</v>
       </c>
       <c r="E17" t="str">
-        <v>Kids Girls Party Frock, Age 5Y</v>
+        <v>Mens Casual Slippers Blue Size 9</v>
       </c>
       <c r="F17">
-        <v>429</v>
+        <v>349</v>
       </c>
       <c r="G17">
-        <v>37.6</v>
+        <v>32.64</v>
       </c>
       <c r="H17">
-        <v>48.57</v>
+        <v>41.44</v>
       </c>
       <c r="I17">
         <v>0</v>
       </c>
       <c r="J17">
-        <v>0.43</v>
+        <v>0.35</v>
       </c>
       <c r="K17">
-        <v>342.4</v>
+        <v>274.57</v>
       </c>
       <c r="L17" t="str">
         <v>Delivered</v>
@@ -1098,37 +1098,37 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2345891118</v>
+        <v>MH1019</v>
       </c>
       <c r="B18" t="str">
-        <v>TXN891118JUL26</v>
+        <v>TXNH1019JUL26</v>
       </c>
       <c r="C18" t="str">
-        <v>07/07/2026</v>
+        <v>09/07/2026</v>
       </c>
       <c r="D18" t="str">
-        <v>ACC-WTCH-BLK</v>
+        <v>FTW-SLPR-BLU-9</v>
       </c>
       <c r="E18" t="str">
-        <v>Analog Wrist Watch - Black Dial</v>
+        <v>Mens Casual Slippers Blue Size 9</v>
       </c>
       <c r="F18">
-        <v>399</v>
+        <v>349</v>
       </c>
       <c r="G18">
-        <v>35.74</v>
+        <v>32.64</v>
       </c>
       <c r="H18">
-        <v>45.07</v>
+        <v>55.03</v>
       </c>
       <c r="I18">
         <v>0</v>
       </c>
       <c r="J18">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
       <c r="K18">
-        <v>317.79</v>
+        <v>215.98</v>
       </c>
       <c r="L18" t="str">
         <v>Delivered</v>
@@ -1139,13 +1139,13 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2345891119</v>
+        <v>MH1020</v>
       </c>
       <c r="B19" t="str">
-        <v>TXN891119JUL26</v>
+        <v>TXNH1020JUL26</v>
       </c>
       <c r="C19" t="str">
-        <v>09/07/2026</v>
+        <v>11/07/2026</v>
       </c>
       <c r="D19" t="str">
         <v>WMN-KRT-YLW-XL</v>
@@ -1160,7 +1160,7 @@
         <v>45.04</v>
       </c>
       <c r="H19">
-        <v>41.04</v>
+        <v>50.32</v>
       </c>
       <c r="I19">
         <v>0</v>
@@ -1169,7 +1169,7 @@
         <v>0.55</v>
       </c>
       <c r="K19">
-        <v>439.37</v>
+        <v>453.09</v>
       </c>
       <c r="L19" t="str">
         <v>Delivered</v>
@@ -1180,13 +1180,13 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2345891120</v>
+        <v>MH1021</v>
       </c>
       <c r="B20" t="str">
-        <v>TXN891120JUL26</v>
+        <v>TXNH1021JUL26</v>
       </c>
       <c r="C20" t="str">
-        <v>11/07/2026</v>
+        <v>13/07/2026</v>
       </c>
       <c r="D20" t="str">
         <v>WMN-KRT-YLW-XL</v>
@@ -1201,7 +1201,7 @@
         <v>45.04</v>
       </c>
       <c r="H20">
-        <v>49.33</v>
+        <v>47.91</v>
       </c>
       <c r="I20">
         <v>0</v>
@@ -1210,7 +1210,7 @@
         <v>0.55</v>
       </c>
       <c r="K20">
-        <v>454.08</v>
+        <v>455.5</v>
       </c>
       <c r="L20" t="str">
         <v>Delivered</v>
@@ -1221,37 +1221,37 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2345891122</v>
+        <v>MH1022</v>
       </c>
       <c r="B21" t="str">
-        <v>TXN891122JUL26</v>
+        <v>TXNH1022JUL26</v>
       </c>
       <c r="C21" t="str">
         <v>15/07/2026</v>
       </c>
       <c r="D21" t="str">
-        <v>ACC-WTCH-BLK</v>
+        <v>WMN-KRT-YLW-XL</v>
       </c>
       <c r="E21" t="str">
-        <v>Analog Wrist Watch - Black Dial</v>
+        <v>Womens Rayon Kurti - Yellow XL</v>
       </c>
       <c r="F21">
-        <v>399</v>
+        <v>549</v>
       </c>
       <c r="G21">
-        <v>35.74</v>
+        <v>45.04</v>
       </c>
       <c r="H21">
-        <v>53.19</v>
+        <v>44.48</v>
       </c>
       <c r="I21">
         <v>0</v>
       </c>
       <c r="J21">
-        <v>0.4</v>
+        <v>0.55</v>
       </c>
       <c r="K21">
-        <v>309.67</v>
+        <v>458.93</v>
       </c>
       <c r="L21" t="str">
         <v>Delivered</v>
@@ -1262,10 +1262,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2345891123</v>
+        <v>MH1023</v>
       </c>
       <c r="B22" t="str">
-        <v>TXN891123JUL26</v>
+        <v>TXNH1023JUL26</v>
       </c>
       <c r="C22" t="str">
         <v>17/07/2026</v>
@@ -1283,7 +1283,7 @@
         <v>85.34</v>
       </c>
       <c r="H22">
-        <v>53.54</v>
+        <v>42.4</v>
       </c>
       <c r="I22">
         <v>0</v>
@@ -1292,7 +1292,7 @@
         <v>1.2</v>
       </c>
       <c r="K22">
-        <v>1058.92</v>
+        <v>1070.06</v>
       </c>
       <c r="L22" t="str">
         <v>Delivered</v>
@@ -1303,37 +1303,37 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2345891124</v>
+        <v>MH1001X</v>
       </c>
       <c r="B23" t="str">
-        <v>TXN891124JUL26</v>
+        <v>TXN1001XJUL26</v>
       </c>
       <c r="C23" t="str">
-        <v>19/07/2026</v>
+        <v>03/07/2026</v>
       </c>
       <c r="D23" t="str">
-        <v>MEN-TRS-DNM-32</v>
+        <v>SAR-BNJ-RED</v>
       </c>
       <c r="E23" t="str">
-        <v>Mens Denim Jeans Slim Fit 32</v>
+        <v>Banarasi Silk Saree - Red</v>
       </c>
       <c r="F23">
-        <v>899</v>
+        <v>1199</v>
       </c>
       <c r="G23">
-        <v>66.74</v>
+        <v>85.34</v>
       </c>
       <c r="H23">
-        <v>54.77</v>
+        <v>41.17</v>
       </c>
       <c r="I23">
         <v>0</v>
       </c>
       <c r="J23">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="K23">
-        <v>776.59</v>
+        <v>535.65</v>
       </c>
       <c r="L23" t="str">
         <v>Delivered</v>
@@ -1344,622 +1344,48 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2345891125</v>
+        <v>MH1008X</v>
       </c>
       <c r="B24" t="str">
-        <v>TXN891125JUL26</v>
+        <v>TXN1008XJUL26</v>
       </c>
       <c r="C24" t="str">
-        <v>21/07/2026</v>
+        <v>17/07/2026</v>
       </c>
       <c r="D24" t="str">
-        <v>SAR-BNJ-RED</v>
+        <v>KRT-WT-MENS-L</v>
       </c>
       <c r="E24" t="str">
-        <v>Banarasi Silk Saree - Red</v>
+        <v>Cotton Kurta Set - White, Men L</v>
       </c>
       <c r="F24">
-        <v>1199</v>
+        <v>749</v>
       </c>
       <c r="G24">
-        <v>85.34</v>
+        <v>57.44</v>
       </c>
       <c r="H24">
-        <v>53.7</v>
+        <v>53.47</v>
       </c>
       <c r="I24">
         <v>0</v>
       </c>
       <c r="J24">
-        <v>1.2</v>
+        <v>0.75</v>
       </c>
       <c r="K24">
-        <v>1058.76</v>
+        <v>318.67</v>
       </c>
       <c r="L24" t="str">
         <v>Delivered</v>
       </c>
       <c r="M24" t="str">
-        <v>Done</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>2345891126</v>
-      </c>
-      <c r="B25" t="str">
-        <v>TXN891126JUL26</v>
-      </c>
-      <c r="C25" t="str">
-        <v>23/07/2026</v>
-      </c>
-      <c r="D25" t="str">
-        <v>KDS-GRL-FRK-5Y</v>
-      </c>
-      <c r="E25" t="str">
-        <v>Kids Girls Party Frock, Age 5Y</v>
-      </c>
-      <c r="F25">
-        <v>429</v>
-      </c>
-      <c r="G25">
-        <v>37.6</v>
-      </c>
-      <c r="H25">
-        <v>41.26</v>
-      </c>
-      <c r="I25">
-        <v>0</v>
-      </c>
-      <c r="J25">
-        <v>0.43</v>
-      </c>
-      <c r="K25">
-        <v>349.71</v>
-      </c>
-      <c r="L25" t="str">
-        <v>Delivered</v>
-      </c>
-      <c r="M25" t="str">
-        <v>Done</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>2345891127</v>
-      </c>
-      <c r="B26" t="str">
-        <v>TXN891127JUL26</v>
-      </c>
-      <c r="C26" t="str">
-        <v>25/07/2026</v>
-      </c>
-      <c r="D26" t="str">
-        <v>MEN-TRS-DNM-32</v>
-      </c>
-      <c r="E26" t="str">
-        <v>Mens Denim Jeans Slim Fit 32</v>
-      </c>
-      <c r="F26">
-        <v>899</v>
-      </c>
-      <c r="G26">
-        <v>66.74</v>
-      </c>
-      <c r="H26">
-        <v>41.39</v>
-      </c>
-      <c r="I26">
-        <v>0</v>
-      </c>
-      <c r="J26">
-        <v>0.9</v>
-      </c>
-      <c r="K26">
-        <v>753.97</v>
-      </c>
-      <c r="L26" t="str">
-        <v>Delivered</v>
-      </c>
-      <c r="M26" t="str">
-        <v>Done</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>2345891128</v>
-      </c>
-      <c r="B27" t="str">
-        <v>TXN891128JUL26</v>
-      </c>
-      <c r="C27" t="str">
-        <v>27/07/2026</v>
-      </c>
-      <c r="D27" t="str">
-        <v>SAR-BNJ-RED</v>
-      </c>
-      <c r="E27" t="str">
-        <v>Banarasi Silk Saree - Red</v>
-      </c>
-      <c r="F27">
-        <v>1199</v>
-      </c>
-      <c r="G27">
-        <v>85.34</v>
-      </c>
-      <c r="H27">
-        <v>55.06</v>
-      </c>
-      <c r="I27">
-        <v>0</v>
-      </c>
-      <c r="J27">
-        <v>1.2</v>
-      </c>
-      <c r="K27">
-        <v>1057.4</v>
-      </c>
-      <c r="L27" t="str">
-        <v>Return</v>
-      </c>
-      <c r="M27" t="str">
-        <v>Done</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>2345891129</v>
-      </c>
-      <c r="B28" t="str">
-        <v>TXN891129JUL26</v>
-      </c>
-      <c r="C28" t="str">
-        <v>29/07/2026</v>
-      </c>
-      <c r="D28" t="str">
-        <v>SAR-BNJ-RED</v>
-      </c>
-      <c r="E28" t="str">
-        <v>Banarasi Silk Saree - Red</v>
-      </c>
-      <c r="F28">
-        <v>1199</v>
-      </c>
-      <c r="G28">
-        <v>85.34</v>
-      </c>
-      <c r="H28">
-        <v>0</v>
-      </c>
-      <c r="I28">
-        <v>68</v>
-      </c>
-      <c r="J28">
-        <v>1.2</v>
-      </c>
-      <c r="K28">
-        <v>976.46</v>
-      </c>
-      <c r="L28" t="str">
-        <v>RTO</v>
-      </c>
-      <c r="M28" t="str">
-        <v>Done</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>2345891130</v>
-      </c>
-      <c r="B29" t="str">
-        <v>TXN891130JUL26</v>
-      </c>
-      <c r="C29" t="str">
-        <v>02/07/2026</v>
-      </c>
-      <c r="D29" t="str">
-        <v>KDS-GRL-FRK-5Y</v>
-      </c>
-      <c r="E29" t="str">
-        <v>Kids Girls Party Frock, Age 5Y</v>
-      </c>
-      <c r="F29">
-        <v>429</v>
-      </c>
-      <c r="G29">
-        <v>37.6</v>
-      </c>
-      <c r="H29">
-        <v>50.21</v>
-      </c>
-      <c r="I29">
-        <v>0</v>
-      </c>
-      <c r="J29">
-        <v>0.43</v>
-      </c>
-      <c r="K29">
-        <v>340.76</v>
-      </c>
-      <c r="L29" t="str">
-        <v>Delivered</v>
-      </c>
-      <c r="M29" t="str">
-        <v>Done</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v>2345891131</v>
-      </c>
-      <c r="B30" t="str">
-        <v>TXN891131JUL26</v>
-      </c>
-      <c r="C30" t="str">
-        <v>03/07/2026</v>
-      </c>
-      <c r="D30" t="str">
-        <v>HOM-BDSHT-DBL</v>
-      </c>
-      <c r="E30" t="str">
-        <v>Double Bedsheet with 2 Pillow Covers</v>
-      </c>
-      <c r="F30">
-        <v>649</v>
-      </c>
-      <c r="G30">
-        <v>51.24</v>
-      </c>
-      <c r="H30">
-        <v>49.77</v>
-      </c>
-      <c r="I30">
-        <v>0</v>
-      </c>
-      <c r="J30">
-        <v>0.65</v>
-      </c>
-      <c r="K30">
-        <v>547.34</v>
-      </c>
-      <c r="L30" t="str">
-        <v>Delivered</v>
-      </c>
-      <c r="M30" t="str">
-        <v>Done</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>2345891132</v>
-      </c>
-      <c r="B31" t="str">
-        <v>TXN891132JUL26</v>
-      </c>
-      <c r="C31" t="str">
-        <v>05/07/2026</v>
-      </c>
-      <c r="D31" t="str">
-        <v>ACC-WTCH-BLK</v>
-      </c>
-      <c r="E31" t="str">
-        <v>Analog Wrist Watch - Black Dial</v>
-      </c>
-      <c r="F31">
-        <v>399</v>
-      </c>
-      <c r="G31">
-        <v>35.74</v>
-      </c>
-      <c r="H31">
-        <v>50.12</v>
-      </c>
-      <c r="I31">
-        <v>0</v>
-      </c>
-      <c r="J31">
-        <v>0.4</v>
-      </c>
-      <c r="K31">
-        <v>312.74</v>
-      </c>
-      <c r="L31" t="str">
-        <v>Delivered</v>
-      </c>
-      <c r="M31" t="str">
-        <v>Done</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v>2345891133</v>
-      </c>
-      <c r="B32" t="str">
-        <v>TXN891133JUL26</v>
-      </c>
-      <c r="C32" t="str">
-        <v>07/07/2026</v>
-      </c>
-      <c r="D32" t="str">
-        <v>WMN-KRT-YLW-XL</v>
-      </c>
-      <c r="E32" t="str">
-        <v>Womens Rayon Kurti - Yellow XL</v>
-      </c>
-      <c r="F32">
-        <v>549</v>
-      </c>
-      <c r="G32">
-        <v>45.04</v>
-      </c>
-      <c r="H32">
-        <v>42.33</v>
-      </c>
-      <c r="I32">
-        <v>0</v>
-      </c>
-      <c r="J32">
-        <v>0.55</v>
-      </c>
-      <c r="K32">
-        <v>461.08</v>
-      </c>
-      <c r="L32" t="str">
-        <v>Delivered</v>
-      </c>
-      <c r="M32" t="str">
-        <v>Done</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>2345891134</v>
-      </c>
-      <c r="B33" t="str">
-        <v>TXN891134JUL26</v>
-      </c>
-      <c r="C33" t="str">
-        <v>09/07/2026</v>
-      </c>
-      <c r="D33" t="str">
-        <v>KDS-GRL-FRK-5Y</v>
-      </c>
-      <c r="E33" t="str">
-        <v>Kids Girls Party Frock, Age 5Y</v>
-      </c>
-      <c r="F33">
-        <v>429</v>
-      </c>
-      <c r="G33">
-        <v>37.6</v>
-      </c>
-      <c r="H33">
-        <v>42.2</v>
-      </c>
-      <c r="I33">
-        <v>0</v>
-      </c>
-      <c r="J33">
-        <v>0.43</v>
-      </c>
-      <c r="K33">
-        <v>348.77</v>
-      </c>
-      <c r="L33" t="str">
-        <v>Delivered</v>
-      </c>
-      <c r="M33" t="str">
-        <v>Done</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v>2345891135</v>
-      </c>
-      <c r="B34" t="str">
-        <v>TXN891135JUL26</v>
-      </c>
-      <c r="C34" t="str">
-        <v>11/07/2026</v>
-      </c>
-      <c r="D34" t="str">
-        <v>FTW-SLPR-BLU-9</v>
-      </c>
-      <c r="E34" t="str">
-        <v>Mens Casual Slippers Blue Size 9</v>
-      </c>
-      <c r="F34">
-        <v>349</v>
-      </c>
-      <c r="G34">
-        <v>32.64</v>
-      </c>
-      <c r="H34">
-        <v>55.64</v>
-      </c>
-      <c r="I34">
-        <v>0</v>
-      </c>
-      <c r="J34">
-        <v>0.35</v>
-      </c>
-      <c r="K34">
-        <v>260.37</v>
-      </c>
-      <c r="L34" t="str">
-        <v>Return</v>
-      </c>
-      <c r="M34" t="str">
-        <v>Done</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v>2345891136</v>
-      </c>
-      <c r="B35" t="str">
-        <v>TXN891136JUL26</v>
-      </c>
-      <c r="C35" t="str">
-        <v>13/07/2026</v>
-      </c>
-      <c r="D35" t="str">
-        <v>SAR-BNJ-RED</v>
-      </c>
-      <c r="E35" t="str">
-        <v>Banarasi Silk Saree - Red</v>
-      </c>
-      <c r="F35">
-        <v>1199</v>
-      </c>
-      <c r="G35">
-        <v>85.34</v>
-      </c>
-      <c r="H35">
-        <v>53.21</v>
-      </c>
-      <c r="I35">
-        <v>0</v>
-      </c>
-      <c r="J35">
-        <v>1.2</v>
-      </c>
-      <c r="K35">
-        <v>1059.25</v>
-      </c>
-      <c r="L35" t="str">
-        <v>Delivered</v>
-      </c>
-      <c r="M35" t="str">
-        <v>Done</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>2345891137</v>
-      </c>
-      <c r="B36" t="str">
-        <v>TXN891137JUL26</v>
-      </c>
-      <c r="C36" t="str">
-        <v>15/07/2026</v>
-      </c>
-      <c r="D36" t="str">
-        <v>SAR-BNJ-RED</v>
-      </c>
-      <c r="E36" t="str">
-        <v>Banarasi Silk Saree - Red</v>
-      </c>
-      <c r="F36">
-        <v>1199</v>
-      </c>
-      <c r="G36">
-        <v>85.34</v>
-      </c>
-      <c r="H36">
-        <v>47.33</v>
-      </c>
-      <c r="I36">
-        <v>0</v>
-      </c>
-      <c r="J36">
-        <v>1.2</v>
-      </c>
-      <c r="K36">
-        <v>1065.13</v>
-      </c>
-      <c r="L36" t="str">
-        <v>Delivered</v>
-      </c>
-      <c r="M36" t="str">
-        <v>Done</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <v>2345891101X</v>
-      </c>
-      <c r="B37" t="str">
-        <v>TXN91101XJUL26</v>
-      </c>
-      <c r="C37" t="str">
-        <v>03/07/2026</v>
-      </c>
-      <c r="D37" t="str">
-        <v>WMN-KRT-YLW-XL</v>
-      </c>
-      <c r="E37" t="str">
-        <v>Womens Rayon Kurti - Yellow XL</v>
-      </c>
-      <c r="F37">
-        <v>549</v>
-      </c>
-      <c r="G37">
-        <v>45.04</v>
-      </c>
-      <c r="H37">
-        <v>48.8</v>
-      </c>
-      <c r="I37">
-        <v>0</v>
-      </c>
-      <c r="J37">
-        <v>0.55</v>
-      </c>
-      <c r="K37">
-        <v>454.61</v>
-      </c>
-      <c r="L37" t="str">
-        <v>Delivered</v>
-      </c>
-      <c r="M37" t="str">
-        <v>Done</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="str">
-        <v>2345891102X</v>
-      </c>
-      <c r="B38" t="str">
-        <v>TXN91102XJUL26</v>
-      </c>
-      <c r="C38" t="str">
-        <v>05/07/2026</v>
-      </c>
-      <c r="D38" t="str">
-        <v>FTW-SLPR-BLU-9</v>
-      </c>
-      <c r="E38" t="str">
-        <v>Mens Casual Slippers Blue Size 9</v>
-      </c>
-      <c r="F38">
-        <v>349</v>
-      </c>
-      <c r="G38">
-        <v>32.64</v>
-      </c>
-      <c r="H38">
-        <v>51.48</v>
-      </c>
-      <c r="I38">
-        <v>0</v>
-      </c>
-      <c r="J38">
-        <v>0.35</v>
-      </c>
-      <c r="K38">
-        <v>264.53</v>
-      </c>
-      <c r="L38" t="str">
-        <v>Delivered</v>
-      </c>
-      <c r="M38" t="str">
         <v>Done</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M24"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>